<commit_message>
added father information to the tables
</commit_message>
<xml_diff>
--- a/Ancestors Database_v2_copy.xlsx
+++ b/Ancestors Database_v2_copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD87AC09-45E0-4479-87EE-49EC887B162A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90AC0CF8-05B7-4554-A239-D598693BADFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46185" yWindow="10440" windowWidth="26010" windowHeight="10545" xr2:uid="{0C8A6B89-EB97-4AFD-AB2D-26665E6E306C}"/>
+    <workbookView xWindow="46110" yWindow="0" windowWidth="26085" windowHeight="20985" xr2:uid="{0C8A6B89-EB97-4AFD-AB2D-26665E6E306C}"/>
   </bookViews>
   <sheets>
     <sheet name="Brooker" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="244">
   <si>
     <t>First Name</t>
   </si>
@@ -766,6 +766,12 @@
   </si>
   <si>
     <t>Spouse_Gen_1_Death_Date</t>
+  </si>
+  <si>
+    <t>Father_FirstName</t>
+  </si>
+  <si>
+    <t>Father_Surname</t>
   </si>
 </sst>
 </file>
@@ -947,7 +953,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1131,6 +1137,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1475,7 +1484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DE48D45-AEF7-4792-8B25-51210844ABFF}">
-  <dimension ref="A1:AB30"/>
+  <dimension ref="A1:AD34"/>
   <sheetFormatPr defaultColWidth="19.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
@@ -1506,9 +1515,11 @@
     <col min="26" max="26" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="59" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="59" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="55" t="s">
         <v>231</v>
       </c>
@@ -1593,8 +1604,14 @@
       <c r="AB1" s="56" t="s">
         <v>241</v>
       </c>
+      <c r="AC1" s="64" t="s">
+        <v>242</v>
+      </c>
+      <c r="AD1" s="64" t="s">
+        <v>243</v>
+      </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>44</v>
       </c>
@@ -1678,7 +1695,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="62"/>
       <c r="B3" s="62"/>
       <c r="C3" s="62"/>
@@ -1696,7 +1713,7 @@
       <c r="R3" s="62"/>
       <c r="S3" s="62"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>49</v>
       </c>
@@ -1765,8 +1782,14 @@
       <c r="AA4" s="61" t="s">
         <v>29</v>
       </c>
+      <c r="AC4" s="60" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD4" s="60" t="s">
+        <v>45</v>
+      </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="60" t="s">
         <v>46</v>
       </c>
@@ -1835,12 +1858,18 @@
       <c r="AA5" s="61" t="s">
         <v>29</v>
       </c>
+      <c r="AC5" s="60" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD5" s="60" t="s">
+        <v>45</v>
+      </c>
     </row>
-    <row r="6" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="F6"/>
       <c r="I6"/>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="60" t="s">
         <v>52</v>
       </c>
@@ -1903,8 +1932,14 @@
       <c r="AA7" s="61" t="s">
         <v>29</v>
       </c>
+      <c r="AC7" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD7" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
         <v>54</v>
       </c>
@@ -1971,8 +2006,14 @@
       <c r="AA8" s="61" t="s">
         <v>29</v>
       </c>
+      <c r="AC8" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD8" s="60" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="60" t="s">
         <v>57</v>
       </c>
@@ -2033,8 +2074,14 @@
       <c r="AA9" s="61" t="s">
         <v>29</v>
       </c>
+      <c r="AC9" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD9" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="60" t="s">
         <v>58</v>
       </c>
@@ -2082,12 +2129,18 @@
       <c r="AA10" s="61" t="s">
         <v>29</v>
       </c>
+      <c r="AC10" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD10" s="60" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="11" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="F11"/>
       <c r="I11"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="60" t="s">
         <v>59</v>
       </c>
@@ -2126,8 +2179,14 @@
       <c r="Q12" s="60"/>
       <c r="R12" s="60"/>
       <c r="S12" s="60"/>
+      <c r="AC12" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD12" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="60" t="s">
         <v>62</v>
       </c>
@@ -2166,8 +2225,14 @@
       <c r="Q13" s="60"/>
       <c r="R13" s="60"/>
       <c r="S13" s="60"/>
+      <c r="AC13" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD13" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="60" t="s">
         <v>65</v>
       </c>
@@ -2210,8 +2275,14 @@
       <c r="R14" t="s">
         <v>35</v>
       </c>
+      <c r="AC14" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD14" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="60" t="s">
         <v>67</v>
       </c>
@@ -2248,8 +2319,14 @@
       <c r="Q15" s="60"/>
       <c r="R15" s="60"/>
       <c r="S15" s="60"/>
+      <c r="AC15" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD15" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="60" t="s">
         <v>69</v>
       </c>
@@ -2286,8 +2363,14 @@
       <c r="Q16" s="60"/>
       <c r="R16" s="60"/>
       <c r="S16" s="60"/>
+      <c r="AC16" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD16" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="60" t="s">
         <v>71</v>
       </c>
@@ -2324,8 +2407,14 @@
       <c r="Q17" s="60"/>
       <c r="R17" s="60"/>
       <c r="S17" s="60"/>
+      <c r="AC17" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD17" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="60" t="s">
         <v>73</v>
       </c>
@@ -2362,8 +2451,14 @@
       <c r="Q18" s="60"/>
       <c r="R18" s="60"/>
       <c r="S18" s="60"/>
+      <c r="AC18" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD18" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="60" t="s">
         <v>75</v>
       </c>
@@ -2400,8 +2495,14 @@
       <c r="Q19" s="60"/>
       <c r="R19" s="60"/>
       <c r="S19" s="60"/>
+      <c r="AC19" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD19" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="60" t="s">
         <v>77</v>
       </c>
@@ -2441,8 +2542,14 @@
       <c r="R20" t="s">
         <v>115</v>
       </c>
+      <c r="AC20" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD20" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="60" t="s">
         <v>79</v>
       </c>
@@ -2484,8 +2591,14 @@
       <c r="R21" t="s">
         <v>117</v>
       </c>
+      <c r="AC21" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD21" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="60" t="s">
         <v>79</v>
       </c>
@@ -2522,8 +2635,14 @@
       <c r="Q22" s="60"/>
       <c r="R22" s="60"/>
       <c r="S22" s="60"/>
+      <c r="AC22" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD22" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="60" t="s">
         <v>83</v>
       </c>
@@ -2562,13 +2681,19 @@
       <c r="Q23" s="60"/>
       <c r="R23" s="60"/>
       <c r="S23" s="60"/>
+      <c r="AC23" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD23" s="60" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="24" spans="1:19" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19"/>
       <c r="F24"/>
       <c r="I24"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="61" t="s">
         <v>118</v>
       </c>
@@ -2616,8 +2741,14 @@
       <c r="Q25" s="61"/>
       <c r="R25" s="60"/>
       <c r="S25" s="60"/>
+      <c r="AC25" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD25" s="60" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="61" t="s">
         <v>89</v>
       </c>
@@ -2657,8 +2788,14 @@
       <c r="R26" t="s">
         <v>121</v>
       </c>
+      <c r="AC26" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD26" s="60" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61" t="s">
         <v>91</v>
       </c>
@@ -2698,8 +2835,14 @@
       <c r="R27" t="s">
         <v>122</v>
       </c>
+      <c r="AC27" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD27" s="60" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="61" t="s">
         <v>93</v>
       </c>
@@ -2739,8 +2882,14 @@
       <c r="R28" t="s">
         <v>35</v>
       </c>
+      <c r="AC28" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD28" s="60" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61" t="s">
         <v>94</v>
       </c>
@@ -2775,8 +2924,14 @@
       <c r="O29" s="61"/>
       <c r="P29" s="61"/>
       <c r="Q29" s="60"/>
+      <c r="AC29" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD29" s="60" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="61" t="s">
         <v>96</v>
       </c>
@@ -2815,6 +2970,41 @@
       </c>
       <c r="R30" t="s">
         <v>126</v>
+      </c>
+      <c r="AC30" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD30" s="60" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AC31" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD31" s="60" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="AC32" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD32" s="60" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="29:30" x14ac:dyDescent="0.25">
+      <c r="AC33" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD33" s="60" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="29:30" x14ac:dyDescent="0.25">
+      <c r="AC34" s="60" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cleaned the book of negroes records and got coordinates for connecticut_state soldiers
</commit_message>
<xml_diff>
--- a/Ancestors Database_v2_copy.xlsx
+++ b/Ancestors Database_v2_copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90AC0CF8-05B7-4554-A239-D598693BADFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F8590C-5C3E-4720-84F4-06B34764C30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46110" yWindow="0" windowWidth="26085" windowHeight="20985" xr2:uid="{0C8A6B89-EB97-4AFD-AB2D-26665E6E306C}"/>
+    <workbookView xWindow="46110" yWindow="0" windowWidth="26085" windowHeight="10545" xr2:uid="{0C8A6B89-EB97-4AFD-AB2D-26665E6E306C}"/>
   </bookViews>
   <sheets>
     <sheet name="Brooker" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="244">
   <si>
     <t>First Name</t>
   </si>
@@ -2979,33 +2979,19 @@
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AC31" s="60" t="s">
-        <v>54</v>
-      </c>
-      <c r="AD31" s="60" t="s">
-        <v>55</v>
-      </c>
+      <c r="AC31" s="60"/>
+      <c r="AD31" s="60"/>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AC32" s="60" t="s">
-        <v>54</v>
-      </c>
-      <c r="AD32" s="60" t="s">
-        <v>55</v>
-      </c>
+      <c r="AC32" s="60"/>
+      <c r="AD32" s="60"/>
     </row>
     <row r="33" spans="29:30" x14ac:dyDescent="0.25">
-      <c r="AC33" s="60" t="s">
-        <v>54</v>
-      </c>
-      <c r="AD33" s="60" t="s">
-        <v>55</v>
-      </c>
+      <c r="AC33" s="60"/>
+      <c r="AD33" s="60"/>
     </row>
     <row r="34" spans="29:30" x14ac:dyDescent="0.25">
-      <c r="AC34" s="60" t="s">
-        <v>54</v>
-      </c>
+      <c r="AC34" s="60"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AB1" xr:uid="{3DE48D45-AEF7-4792-8B25-51210844ABFF}"/>

</xml_diff>